<commit_message>
enhance graticule configuration and UTM zone handling; add independent tick density for axes
</commit_message>
<xml_diff>
--- a/data/mapmaker.xlsx
+++ b/data/mapmaker.xlsx
@@ -23322,7 +23322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23343,7 +23343,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>author</t>
@@ -23356,7 +23360,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>date</t>
@@ -23369,7 +23377,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>attribution.text</t>
@@ -23382,7 +23394,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>company.name</t>
@@ -23395,7 +23411,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>company.logo_path</t>
@@ -23408,7 +23428,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>company.logo_scale</t>
@@ -23419,25 +23443,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>basemap.zoom_adjust</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
+          <t>map.crs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EPSG:4326</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>graticule.hemisphere_labels</t>
-        </is>
-      </c>
-      <c r="C9" t="b">
-        <v>0</v>
+          <t>map.figsize</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>13, 8</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -23448,13 +23484,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>export.filename</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>wind_farm_locations.png</t>
-        </is>
+          <t>map.dpi</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -23465,12 +23499,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>inset_map.location</t>
+          <t>map.background_color</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>upper left</t>
+          <t>white</t>
         </is>
       </c>
     </row>
@@ -23482,13 +23516,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>style.marker</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+          <t>map.padding_fraction</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="13">
@@ -23499,13 +23531,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>style.color</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>#2166ac</t>
-        </is>
+          <t>basemap.show</t>
+        </is>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -23516,12 +23546,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>style.size_field</t>
+          <t>basemap.provider</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>capacity_mw</t>
+          <t>OpenStreetMap.Mapnik</t>
         </is>
       </c>
     </row>
@@ -23533,11 +23563,13 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>style.base_marker_size</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>45</v>
+          <t>basemap.zoom</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -23548,11 +23580,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>style.size_scale</t>
+          <t>basemap.zoom_adjust</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -23563,133 +23595,131 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>style.label_points</t>
-        </is>
-      </c>
-      <c r="C17" t="b">
+          <t>basemap.alpha</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>export.filename</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>turbines.png</t>
-        </is>
+          <t>graticule.show</t>
+        </is>
+      </c>
+      <c r="C18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>map.padding_fraction</t>
+          <t>graticule.n_ticks</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>inset_map.zoom_out_factor</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>40</v>
+          <t>graticule.format</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>inset_map.size</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0.16</v>
+          <t>graticule.hemisphere_labels</t>
+        </is>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>style.marker</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+          <t>graticule.fontsize</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>style.color</t>
+          <t>graticule.color</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>#2166ac</t>
+          <t>0.35</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>style.marker_size</t>
+          <t>graticule.linewidth</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>55</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>style.label_points</t>
+          <t>graticule.frame</t>
         </is>
       </c>
       <c r="C25" t="b">
@@ -23699,222 +23729,2192 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>graticule.n_ticks</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
+          <t>legend.show</t>
+        </is>
+      </c>
+      <c r="C26" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>export.filename</t>
+          <t>legend.title</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>era5_merra2_grid_cells.png</t>
+          <t>Legend</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>map.padding_fraction</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0.05</v>
+          <t>scalebar.show</t>
+        </is>
+      </c>
+      <c r="C28" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inset_map.zoom_out_factor</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>4</v>
+          <t>scalebar.units</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>inset_map.size</t>
+          <t>scalebar.length_fraction</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.22</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>north_arrow.size</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>0.035</v>
+          <t>north_arrow.show</t>
+        </is>
+      </c>
+      <c r="C31" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>style.marker</t>
+          <t>north_arrow.location</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>lower right</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>style.dataset_markers.ERA5</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+          <t>north_arrow.size</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.045</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>style.dataset_markers.MERRA2</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+          <t>inset_map.show</t>
+        </is>
+      </c>
+      <c r="C34" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>style.dataset_colors.ERA5</t>
+          <t>inset_map.location</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>#3182bd</t>
+          <t>upper left</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>style.dataset_colors.MERRA2</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>#e6550d</t>
-        </is>
+          <t>inset_map.size</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>style.marker_size</t>
+          <t>inset_map.zoom_out_factor</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>wind_farms</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>graticule.n_ticks</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>6</v>
+          <t>inset_map.bbox_edgecolor</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>inset_map.bbox_linewidth</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>inset_map.min_bbox_frac</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>footer.show</t>
+        </is>
+      </c>
+      <c r="C41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>footer.height_fraction</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>footer.column_widths</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1.0, 1.3, 1.4, 2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>footer.fontsize</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>footer.text_color</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>export.output_dir</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>../output</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>export.transparent</t>
+        </is>
+      </c>
+      <c r="C47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>export.filename</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>wind_farm_locations.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>style.marker</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>style.color</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>#2166ac</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>style.size_field</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>capacity_mw</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>style.base_marker_size</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>style.size_scale</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>style.label_points</t>
+        </is>
+      </c>
+      <c r="C54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>wind_farms</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>style.declutter_labels</t>
+        </is>
+      </c>
+      <c r="C55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Yash Mahajan</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>attribution.text</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>© OpenStreetMap (OSM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>company.name</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>DNV Energy Systems Germany GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>company.logo_path</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>../assets/logo.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>company.logo_scale</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>map.crs</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>EPSG:4326</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>map.figsize</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>13, 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>map.dpi</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>map.background_color</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>map.padding_fraction</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>basemap.show</t>
+        </is>
+      </c>
+      <c r="C67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>basemap.provider</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>OpenStreetMap.Mapnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>basemap.zoom</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>basemap.zoom_adjust</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>basemap.alpha</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>graticule.show</t>
+        </is>
+      </c>
+      <c r="C72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>graticule.n_ticks</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>graticule.format</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>graticule.hemisphere_labels</t>
+        </is>
+      </c>
+      <c r="C75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>graticule.fontsize</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>graticule.color</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>graticule.linewidth</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>graticule.frame</t>
+        </is>
+      </c>
+      <c r="C79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>legend.show</t>
+        </is>
+      </c>
+      <c r="C80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>legend.title</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>scalebar.show</t>
+        </is>
+      </c>
+      <c r="C82" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>scalebar.units</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>scalebar.length_fraction</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>north_arrow.show</t>
+        </is>
+      </c>
+      <c r="C85" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>north_arrow.location</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>lower right</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>north_arrow.size</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>inset_map.show</t>
+        </is>
+      </c>
+      <c r="C88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>inset_map.location</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>lower left</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>inset_map.size</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>inset_map.zoom_out_factor</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>inset_map.bbox_edgecolor</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>inset_map.bbox_linewidth</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>inset_map.min_bbox_frac</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>footer.show</t>
+        </is>
+      </c>
+      <c r="C95" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>footer.height_fraction</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>footer.column_widths</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>1.0, 1.3, 1.4, 2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>footer.fontsize</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>footer.text_color</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>export.output_dir</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>../output</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>export.transparent</t>
+        </is>
+      </c>
+      <c r="C101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>export.filename</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>turbines.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>style.marker</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>style.color</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>#2166ac</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>style.marker_size</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>style.label_points</t>
+        </is>
+      </c>
+      <c r="C106" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>turbines</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>style.declutter_labels</t>
+        </is>
+      </c>
+      <c r="C107" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
           <t>grid_cells</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Yash Mahajan</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>attribution.text</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>© OpenStreetMap (OSM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>company.name</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>DNV Energy Systems Germany GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>company.logo_path</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>../assets/logo.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>company.logo_scale</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>map.crs</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>EPSG:4326</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>map.figsize</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>13, 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>map.dpi</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>map.background_color</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>map.padding_fraction</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>basemap.show</t>
+        </is>
+      </c>
+      <c r="C119" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>basemap.provider</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>OpenStreetMap.Mapnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>basemap.zoom</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>basemap.zoom_adjust</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>basemap.alpha</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>graticule.show</t>
+        </is>
+      </c>
+      <c r="C124" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>graticule.n_ticks</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>graticule.format</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>graticule.hemisphere_labels</t>
+        </is>
+      </c>
+      <c r="C127" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>graticule.fontsize</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>graticule.color</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>graticule.linewidth</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>graticule.frame</t>
+        </is>
+      </c>
+      <c r="C131" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>legend.show</t>
+        </is>
+      </c>
+      <c r="C132" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>legend.title</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>scalebar.show</t>
+        </is>
+      </c>
+      <c r="C134" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>scalebar.units</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>scalebar.length_fraction</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>north_arrow.show</t>
+        </is>
+      </c>
+      <c r="C137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>north_arrow.location</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>lower right</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>north_arrow.size</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>inset_map.show</t>
+        </is>
+      </c>
+      <c r="C140" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>inset_map.location</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>lower left</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>inset_map.size</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>inset_map.zoom_out_factor</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>inset_map.bbox_edgecolor</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>inset_map.bbox_linewidth</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>inset_map.min_bbox_frac</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>footer.show</t>
+        </is>
+      </c>
+      <c r="C147" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>footer.height_fraction</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>footer.column_widths</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>1.0, 1.3, 1.4, 2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>footer.fontsize</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>footer.text_color</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>export.output_dir</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>../output</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>export.transparent</t>
+        </is>
+      </c>
+      <c r="C153" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>export.filename</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>era5_merra2_grid_cells.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>style.marker</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>style.dataset_markers.ERA5</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>style.dataset_markers.MERRA2</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>style.dataset_colors.ERA5</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>#3182bd</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>style.dataset_colors.MERRA2</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>#e6550d</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>style.marker_size</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>graticule.n_ticks_x</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>graticule.n_ticks_y</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>grid_cells</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
         <is>
           <t>reference_point.show</t>
         </is>
       </c>
-      <c r="C39" t="b">
+      <c r="C163" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor map configuration for improved readability and compatibility; update timeout handling for basemap requests
</commit_message>
<xml_diff>
--- a/data/mapmaker.xlsx
+++ b/data/mapmaker.xlsx
@@ -25063,7 +25063,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -25278,7 +25278,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dotted path into contextily.providers. Try "CartoDB.Positron"/"Esri.WorldGrayCanvas" for a muted look, or "Esri.WorldShadedRelief"/"OpenTopoMap"/"Esri.WorldTopoMap" for a terrain/relief basemap.</t>
+          <t>Dotted path into contextily.providers. Try "CartoDB.Positron"/"Esri.WorldGrayCanvas" for a muted look, or "Esri.WorldShadedRelief"/"OpenTopoMap"/"Esri.WorldTopoMap" for a terrain/relief basemap. A full URL template containing {x}/{y}/{z} (e.g. a Mapbox/Google/private tile URL with your own API key already embedded) is also accepted and used as-is instead of being looked up in contextily.providers.</t>
         </is>
       </c>
     </row>
@@ -25399,7 +25399,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -25419,7 +25419,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -25439,7 +25439,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -25459,7 +25459,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -25481,7 +25481,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -25503,7 +25503,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -25525,7 +25525,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -25547,7 +25547,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -25567,7 +25567,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -25587,7 +25587,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -25607,7 +25607,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -25627,7 +25627,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -25649,7 +25649,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -25671,7 +25671,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -25693,7 +25693,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -25715,7 +25715,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -25737,7 +25737,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -25759,7 +25759,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -25781,7 +25781,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -25803,7 +25803,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -25825,7 +25825,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -25847,7 +25847,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>wind_farms</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -25869,7 +25869,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -25891,7 +25891,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -25913,7 +25913,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -25933,7 +25933,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -25953,7 +25953,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -25973,7 +25973,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -25995,7 +25995,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -26017,7 +26017,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -26039,7 +26039,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -26061,7 +26061,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -26083,7 +26083,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -26105,7 +26105,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -26127,7 +26127,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -26149,7 +26149,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -26171,7 +26171,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -26193,7 +26193,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -26213,7 +26213,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -26233,7 +26233,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -26261,13 +26261,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -26432,7 +26432,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>HTTP header sent with tile requests -- OSM requires a descriptive User-Agent or it silently serves a "blocked" placeholder tile. Replace the contact email before heavy/production use.</t>
+          <t>HTTP header sent with tile requests -- OSM enforces this and will serve a visible "Access blocked" tile (not a silent failure) for a generic/placeholder User-Agent. Replace the contact email before heavy/production use.</t>
         </is>
       </c>
     </row>
@@ -26440,17 +26440,15 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>basemap.interpolation</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>bilinear</t>
-        </is>
+          <t>basemap.timeout</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>How the basemap's fixed-resolution tile pixels are resampled up to the map panel's print size. Try "lanczos" for crisper-looking tile text/lines at high dpi (at some risk of ringing artifacts on hard edges) -- raising basemap.zoom_adjust helps more, since it fetches genuinely more detailed tiles instead of just resampling the same ones.</t>
+          <t>Seconds to wait for a tile server to respond before giving up on that tile. Without this, an unresponsive/rate-limiting server (some free providers throttle or silently drop requests from datacenter/cloud IPs) can hang the whole render indefinitely instead of falling back to a flat fill; lower for faster failover, raise on a slow connection.</t>
         </is>
       </c>
     </row>
@@ -26458,15 +26456,17 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>graticule.n_ticks</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>5</v>
+          <t>basemap.interpolation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>bilinear</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Approximate number of tick/cross lines per axis; shared fallback for both axes when n_ticks_x/n_ticks_y aren't set.</t>
+          <t>How the basemap's fixed-resolution tile pixels are resampled up to the map panel's print size. Try "lanczos" for crisper-looking tile text/lines at high dpi (at some risk of ringing artifacts on hard edges) -- raising basemap.zoom_adjust helps more, since it fetches genuinely more detailed tiles instead of just resampling the same ones.</t>
         </is>
       </c>
     </row>
@@ -26474,13 +26474,15 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>graticule.n_ticks_x</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>graticule.n_ticks</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Horizontal-axis tick density, independent of the vertical axis. Falls back to graticule.n_ticks if unset.</t>
+          <t>Approximate number of tick/cross lines per axis; shared fallback for both axes when n_ticks_x/n_ticks_y aren't set.</t>
         </is>
       </c>
     </row>
@@ -26488,13 +26490,13 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>graticule.n_ticks_y</t>
+          <t>graticule.n_ticks_x</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Vertical-axis tick density, independent of the horizontal axis. Falls back to graticule.n_ticks if unset.</t>
+          <t>Horizontal-axis tick density, independent of the vertical axis. Falls back to graticule.n_ticks if unset.</t>
         </is>
       </c>
     </row>
@@ -26502,17 +26504,13 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>graticule.format</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
+          <t>graticule.n_ticks_y</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>decimal (e.g. 5.90°) or dms (degrees/minutes/seconds, e.g. 5°54'00.0"). Only applies when map.crs is geographic (e.g. the default EPSG:4326) -- a projected CRS like UTM always shows native-unit (meter) ticks instead.</t>
+          <t>Vertical-axis tick density, independent of the horizontal axis. Falls back to graticule.n_ticks if unset.</t>
         </is>
       </c>
     </row>
@@ -26520,15 +26518,17 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>graticule.hemisphere_labels</t>
-        </is>
-      </c>
-      <c r="C16" t="b">
-        <v>0</v>
+          <t>graticule.format</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>true appends E/N/W/S; false drops the letter and keeps a "-" sign for west/south instead.</t>
+          <t>decimal (e.g. 5.90°) or dms (degrees/minutes/seconds, e.g. 5°54'00.0"). Only applies when map.crs is geographic (e.g. the default EPSG:4326) -- a projected CRS like UTM always shows native-unit (meter) ticks instead.</t>
         </is>
       </c>
     </row>
@@ -26536,15 +26536,15 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>graticule.fontsize</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>10</v>
+          <t>graticule.hemisphere_labels</t>
+        </is>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tick label font size.</t>
+          <t>true appends E/N/W/S; false drops the letter and keeps a "-" sign for west/south instead.</t>
         </is>
       </c>
     </row>
@@ -26552,17 +26552,15 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>graticule.color</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>0.35</t>
-        </is>
+          <t>graticule.fontsize</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Tick/cross mark color.</t>
+          <t>Tick label font size.</t>
         </is>
       </c>
     </row>
@@ -26570,15 +26568,17 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>graticule.linewidth</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>0.6</v>
+          <t>graticule.color</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Tick/cross mark line width.</t>
+          <t>Tick/cross mark color.</t>
         </is>
       </c>
     </row>
@@ -26586,15 +26586,15 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>graticule.frame</t>
-        </is>
-      </c>
-      <c r="C20" t="b">
-        <v>1</v>
+          <t>graticule.linewidth</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Draw the black frame/spines around the map panel.</t>
+          <t>Tick/cross mark line width.</t>
         </is>
       </c>
     </row>
@@ -26602,17 +26602,15 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>scalebar.units</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
+          <t>graticule.frame</t>
+        </is>
+      </c>
+      <c r="C21" t="b">
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>auto (m below 1 km, else km), or force m/km.</t>
+          <t>Draw the black frame/spines around the map panel.</t>
         </is>
       </c>
     </row>
@@ -26620,15 +26618,17 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>scalebar.length_fraction</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>0.55</v>
+          <t>scalebar.units</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Target fraction of the scale bar panel's width the bar should roughly fill before rounding to a nice number.</t>
+          <t>auto (m below 1 km, else km), or force m/km.</t>
         </is>
       </c>
     </row>
@@ -26636,17 +26636,15 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>north_arrow.location</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>lower right</t>
-        </is>
+          <t>scalebar.length_fraction</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.55</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Corner inside the map frame: upper left/upper right/lower left/lower right.</t>
+          <t>Target fraction of the scale bar panel's width the bar should roughly fill before rounding to a nice number.</t>
         </is>
       </c>
     </row>
@@ -26654,15 +26652,17 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>north_arrow.size</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0.045</v>
+          <t>north_arrow.location</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>lower right</t>
+        </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arrow size, as a fraction of the map panel.</t>
+          <t>Corner inside the map frame: upper left/upper right/lower left/lower right.</t>
         </is>
       </c>
     </row>
@@ -26670,17 +26670,15 @@
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>inset_map.location</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>lower left</t>
-        </is>
+          <t>north_arrow.size</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.045</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Corner inside the map frame (same 4 options as north_arrow.location).</t>
+          <t>Arrow size, as a fraction of the map panel.</t>
         </is>
       </c>
     </row>
@@ -26688,15 +26686,17 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>inset_map.size</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0.28</v>
+          <t>inset_map.location</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>lower left</t>
+        </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Inset size as a fraction of the map panel.</t>
+          <t>Corner inside the map frame (same 4 options as north_arrow.location).</t>
         </is>
       </c>
     </row>
@@ -26704,15 +26704,15 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>inset_map.zoom_out_factor</t>
+          <t>inset_map.size</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>0.28</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>How many times wider/taller the inset's view is than the main map's extent.</t>
+          <t>Inset size as a fraction of the map panel.</t>
         </is>
       </c>
     </row>
@@ -26720,17 +26720,15 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>inset_map.bbox_edgecolor</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
+          <t>inset_map.zoom_out_factor</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Color of the ROI bounding box drawn on the inset.</t>
+          <t>How many times wider/taller the inset's view is than the main map's extent.</t>
         </is>
       </c>
     </row>
@@ -26738,15 +26736,17 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inset_map.bbox_linewidth</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>2.2</v>
+          <t>inset_map.bbox_edgecolor</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Line width of that ROI bounding box.</t>
+          <t>Color of the ROI bounding box drawn on the inset.</t>
         </is>
       </c>
     </row>
@@ -26754,15 +26754,15 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>inset_map.min_bbox_frac</t>
+          <t>inset_map.bbox_linewidth</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.05</v>
+        <v>2.2</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Floors the ROI box to at least this fraction of the inset's width/height, so it stays visible at a large zoom_out_factor.</t>
+          <t>Line width of that ROI bounding box.</t>
         </is>
       </c>
     </row>
@@ -26770,15 +26770,15 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>footer.height_fraction</t>
+          <t>inset_map.min_bbox_frac</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>How tall the footer band is, as a fraction of the page.</t>
+          <t>Floors the ROI box to at least this fraction of the inset's width/height, so it stays visible at a large zoom_out_factor.</t>
         </is>
       </c>
     </row>
@@ -26786,17 +26786,15 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>footer.column_widths</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1.0, 1.3, 1.4, 2.1</t>
-        </is>
+          <t>footer.height_fraction</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0.09</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Relative widths of the legend / scale bar / CRS / date-author-copyright+logo columns.</t>
+          <t>How tall the footer band is, as a fraction of the page.</t>
         </is>
       </c>
     </row>
@@ -26804,15 +26802,17 @@
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>footer.fontsize</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>8</v>
+          <t>footer.column_widths</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1.0, 1.3, 1.4, 2.1</t>
+        </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Footer text size.</t>
+          <t>Relative widths of the legend / scale bar / CRS / date-author-copyright+logo columns.</t>
         </is>
       </c>
     </row>
@@ -26820,17 +26820,15 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>footer.text_color</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
+          <t>footer.fontsize</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>8</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Footer text color.</t>
+          <t>Footer text size.</t>
         </is>
       </c>
     </row>
@@ -26838,17 +26836,17 @@
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>export.output_dir</t>
+          <t>footer.text_color</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>../output</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Output folder, resolved relative to the workbook's own directory.</t>
+          <t>Footer text color.</t>
         </is>
       </c>
     </row>
@@ -26856,15 +26854,17 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>export.transparent</t>
-        </is>
-      </c>
-      <c r="C36" t="b">
-        <v>0</v>
+          <t>export.output_dir</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>../output</t>
+        </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Export with a transparent background instead of map.background_color.</t>
+          <t>Output folder, resolved relative to the workbook's own directory.</t>
         </is>
       </c>
     </row>
@@ -26872,13 +26872,15 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>data.selected_farm</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>export.transparent</t>
+        </is>
+      </c>
+      <c r="C37" t="b">
+        <v>0</v>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>turbines/grid_cells only: pin the render to one farm_name instead of auto-rendering one map per farm. Leave blank for the auto-split default.</t>
+          <t>Export with a transparent background instead of map.background_color.</t>
         </is>
       </c>
     </row>
@@ -26886,355 +26888,369 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>data.selected_datasets</t>
+          <t>data.selected_farm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
+          <t>turbines/grid_cells only: pin the render to one farm_name instead of auto-rendering one map per farm. Leave blank for the auto-split default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>data.selected_datasets</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>grid_cells only: comma-separated list of dataset values to include; leave blank to render every dataset present.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>wind_farms</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>footer.height_fraction</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Taller than the global 0.09 default -- a 10-entry farm_colors legend needs more vertical room than a short status/uniform legend does.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Portfolio Map</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>map.padding_fraction</t>
+          <t>footer.height_fraction</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.4</v>
+        <v>0.24</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Extra padding around the data extent -- higher than the global default since a turbine grid has no empty margin of its own.</t>
+          <t>Taller than the global 0.09 default -- a 10-entry farm_colors legend needs more vertical room than a short status/uniform legend does.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>inset_map.zoom_out_factor</t>
+          <t>map.padding_fraction</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>40</v>
+        <v>0.4</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Turbine-scale maps need a much larger inset zoom-out than the global default to show useful regional context.</t>
+          <t>Extra padding around the data extent -- higher than the global default since a turbine grid has no empty margin of its own.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>inset_map.size</t>
+          <t>inset_map.zoom_out_factor</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.16</v>
+        <v>40</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Smaller inset than the global default, so it covers less of the tightly-packed turbine layout.</t>
+          <t>Turbine-scale maps need a much larger inset zoom-out than the global default to show useful regional context.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>inset_map.min_bbox_frac</t>
+          <t>inset_map.size</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Raised above the global 0.05 default -- this large a zoom_out_factor would otherwise shrink the true ROI box to a barely-visible sliver.</t>
+          <t>Smaller inset than the global default, so it covers less of the tightly-packed turbine layout.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>turbines</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>graticule.n_ticks</t>
+          <t>inset_map.min_bbox_frac</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>0.12</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fewer ticks than the global default -- a single farm's extent is small enough that 5+ ticks would crowd the frame.</t>
+          <t>Raised above the global 0.05 default -- this large a zoom_out_factor would otherwise shrink the true ROI box to a barely-visible sliver.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>Turbine Map</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>map.padding_fraction</t>
+          <t>graticule.n_ticks</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.05</v>
+        <v>4</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tighter than the global default -- the reanalysis grid already fills its own extent with little empty margin needed.</t>
+          <t>Fewer ticks than the global default -- a single farm's extent is small enough that 5+ ticks would crowd the frame.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>inset_map.zoom_out_factor</t>
+          <t>map.padding_fraction</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>0.05</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Less zoomed-out than the global default -- a regional grid needs less extra context than a single turbine layout does.</t>
+          <t>Tighter than the global default -- the reanalysis grid already fills its own extent with little empty margin needed.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>inset_map.size</t>
+          <t>inset_map.zoom_out_factor</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.22</v>
+        <v>4</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bigger inset than the global default, matching this map's broader regional context.</t>
+          <t>Less zoomed-out than the global default -- a regional grid needs less extra context than a single turbine layout does.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>inset_map.min_bbox_frac</t>
+          <t>inset_map.size</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.08</v>
+        <v>0.22</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Raised above the global 0.05 default for the same visibility reason as turbines, just a smaller bump since zoom_out_factor is lower here.</t>
+          <t>Bigger inset than the global default, matching this map's broader regional context.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>north_arrow.size</t>
+          <t>inset_map.min_bbox_frac</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.035</v>
+        <v>0.08</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Smaller than the global default -- proportionally less obtrusive on this wide regional map.</t>
+          <t>Raised above the global 0.05 default for the same visibility reason as turbines, just a smaller bump since zoom_out_factor is lower here.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>graticule.n_ticks_x</t>
+          <t>north_arrow.size</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>6</v>
+        <v>0.035</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Independent horizontal tick density -- this grid is wider than tall, so a different count than n_ticks_y keeps spacing even on both axes.</t>
+          <t>Smaller than the global default -- proportionally less obtrusive on this wide regional map.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>graticule.n_ticks_y</t>
+          <t>graticule.n_ticks_x</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Independent vertical tick density.</t>
+          <t>Independent horizontal tick density -- this grid is wider than tall, so a different count than n_ticks_y keeps spacing even on both axes.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>reference_point.marker</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+          <t>graticule.n_ticks_y</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Reference point marker shape.</t>
+          <t>Independent vertical tick density.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>reference_point.color</t>
+          <t>reference_point.marker</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>#d62728</t>
+          <t>o</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Reference point marker color.</t>
+          <t>Reference point marker shape.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>reference_point.size</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>70</v>
+          <t>reference_point.color</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>#d62728</t>
+        </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Reference point marker size.</t>
+          <t>Reference point marker color.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>grid_cells</t>
+          <t>ERA5/MERRA2 Map</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>reference_point.size</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>70</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Reference point marker size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ERA5/MERRA2 Map</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>reference_point.label_fontsize</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C56" t="n">
         <v>9</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Reference point label font size.</t>
         </is>

</xml_diff>

<commit_message>
Add packaging support and enhance CLI functionality; include logo asset and update README
</commit_message>
<xml_diff>
--- a/data/mapmaker.xlsx
+++ b/data/mapmaker.xlsx
@@ -12,6 +12,7 @@
     <sheet name="grid_cells" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="settings_basic" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="settings_advanced" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="style_reference" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +30,188 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF696969"/>
+        <bgColor rgb="FF696969"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9A9A9"/>
+        <bgColor rgb="FFA9A9A9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
+        <bgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4682B4"/>
+        <bgColor rgb="FF4682B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4169E1"/>
+        <bgColor rgb="FF4169E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000080"/>
+        <bgColor rgb="FF000080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF87CEEB"/>
+        <bgColor rgb="FF87CEEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF008080"/>
+        <bgColor rgb="FF008080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF008B8B"/>
+        <bgColor rgb="FF008B8B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF228B22"/>
+        <bgColor rgb="FF228B22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E8B57"/>
+        <bgColor rgb="FF2E8B57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808000"/>
+        <bgColor rgb="FF808000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAA520"/>
+        <bgColor rgb="FFDAA520"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD700"/>
+        <bgColor rgb="FFFFD700"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8C00"/>
+        <bgColor rgb="FFFF8C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD2691E"/>
+        <bgColor rgb="FFD2691E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB22222"/>
+        <bgColor rgb="FFB22222"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDC143C"/>
+        <bgColor rgb="FFDC143C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6347"/>
+        <bgColor rgb="FFFF6347"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF800080"/>
+        <bgColor rgb="FF800080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4B0082"/>
+        <bgColor rgb="FF4B0082"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC71585"/>
+        <bgColor rgb="FFC71585"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA52A2A"/>
+        <bgColor rgb="FFA52A2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8B4513"/>
+        <bgColor rgb="FF8B4513"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF708090"/>
+        <bgColor rgb="FF708090"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -50,8 +226,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25210,7 +25419,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Path to the footer logo image, resolved relative to this workbook's own folder.</t>
+          <t>Path to the footer logo image, resolved relative to this workbook's own folder (or use an absolute path). Leave this row out entirely and mapmaker falls back to its own bundled placeholder logo -- see mapmaker/config.py::DEFAULT_LOGO_PATH -- so the footer always shows something even with zero configuration. Set the value to explicitly blank (not just omitting the row) to turn the logo off rather than falling back to the bundled one.</t>
         </is>
       </c>
     </row>
@@ -25518,7 +25727,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Marker shape, any matplotlib marker code ("o" circle, "D" diamond, "^" triangle, ...).</t>
+          <t>Marker shape -- pick from the dropdown, or type any matplotlib marker code (full list: https://matplotlib.org/stable/api/markers_api.html).</t>
         </is>
       </c>
     </row>
@@ -25664,7 +25873,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25686,7 +25895,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25708,7 +25917,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25730,7 +25939,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25752,7 +25961,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25774,7 +25983,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25796,7 +26005,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25818,7 +26027,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25840,7 +26049,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25862,7 +26071,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color.</t>
+          <t>Per-farm color, keyed by the farm's own name -- gives every wind farm its own distinct color and legend entry. Any farm left out of this list falls back to style.color. Kept as exact Okabe-Ito colorblind-safe hex on purpose; the dropdown still offers named colors if you'd rather use one for a farm you add yourself.</t>
         </is>
       </c>
     </row>
@@ -25906,7 +26115,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Marker shape.</t>
+          <t>Marker shape -- pick from the dropdown, or type any matplotlib marker code.</t>
         </is>
       </c>
     </row>
@@ -26010,7 +26219,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Explicit color for one style.color_field category. Any category not listed here still gets colored automatically, cycling through a built-in colorblind-safe palette -- see the next row.</t>
+          <t>Explicit color for one style.color_field category. Kept as an exact Okabe-Ito colorblind-safe hex value on purpose rather than a named color -- the dropdown still offers named alternatives if you'd rather use one. Any category not listed here still gets colored automatically, cycling through the same built-in colorblind-safe palette -- see the next row.</t>
         </is>
       </c>
     </row>
@@ -26076,7 +26285,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Fallback marker shape for any dataset not listed in style.dataset_markers.</t>
+          <t>Fallback marker shape for any dataset not listed in style.dataset_markers -- pick from the dropdown, or type any matplotlib marker code.</t>
         </is>
       </c>
     </row>
@@ -26098,7 +26307,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Per-dataset marker shape override, e.g. "D" diamond, "o" circle, "^" triangle.</t>
+          <t>Per-dataset marker shape override.</t>
         </is>
       </c>
     </row>
@@ -26137,12 +26346,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>#3182bd</t>
+          <t>steelblue</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Per-dataset color.</t>
+          <t>Per-dataset color -- pick from the dropdown (named matplotlib colors, see the style_reference sheet), or type any matplotlib color name/hex code.</t>
         </is>
       </c>
     </row>
@@ -26159,7 +26368,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>#e6550d</t>
+          <t>chocolate</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -26251,6 +26460,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C49 C50 C55 C56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'style_reference'!$A$2:$A$29</formula1>
+    </dataValidation>
+    <dataValidation sqref="C26 C44 C52 C53 C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'style_reference'!$D$2:$D$17</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26334,7 +26551,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Page/figure background color.</t>
+          <t>Page/figure background color -- pick from the dropdown, or type any matplotlib color name/hex code.</t>
         </is>
       </c>
     </row>
@@ -26578,7 +26795,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Tick/cross mark color.</t>
+          <t>Tick/cross mark color. Left as a grayscale intensity (0=black, 1=white) rather than a named color for fine-grained control; the dropdown also offers a few named grays if you'd rather use one.</t>
         </is>
       </c>
     </row>
@@ -26746,7 +26963,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Color of the ROI bounding box drawn on the inset.</t>
+          <t>Color of the ROI bounding box drawn on the inset -- pick from the dropdown, or type any matplotlib color name/hex code.</t>
         </is>
       </c>
     </row>
@@ -26846,7 +27063,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Footer text color.</t>
+          <t>Footer text color. Same grayscale-intensity convention as graticule.color above; the dropdown also offers named grays.</t>
         </is>
       </c>
     </row>
@@ -27190,7 +27407,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Reference point marker shape.</t>
+          <t>Reference point marker shape -- pick from the dropdown, or type any matplotlib marker code (full list: https://matplotlib.org/stable/api/markers_api.html).</t>
         </is>
       </c>
     </row>
@@ -27207,7 +27424,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>#d62728</t>
+          <t>firebrick</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -27257,6 +27474,463 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C4 C19 C29 C35 C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'style_reference'!$A$2:$A$29</formula1>
+    </dataValidation>
+    <dataValidation sqref="C53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'style_reference'!$D$2:$D$17</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Color name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Swatch</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Marker code</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>circle</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dimgray</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>diamond (large)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>darkgray</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>diamond (thin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>lightgray</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>^</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>triangle, pointing up</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>v</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>triangle, pointing down</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>steelblue</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>triangle, pointing left</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>royalblue</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>triangle, pointing right</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>navy</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>pentagon</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>skyblue</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>hexagon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>teal</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>octagon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>darkcyan</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>forestgreen</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>plus (filled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>seagreen</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>x (filled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>olive</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>plus (thin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>goldenrod</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>x (thin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>darkorange</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>chocolate</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>firebrick</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>crimson</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>tomato</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>indigo</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>mediumvioletred</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>brown</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>saddlebrown</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>slategray</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>These lists feed the dropdowns on settings_basic/settings_advanced's "value" column. They're a convenient shortlist, not an exhaustive one -- you can always type any matplotlib color name/hex code or marker code by hand instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Full marker reference:</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>https://matplotlib.org/stable/api/markers_api.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
grid reference fix and gui
</commit_message>
<xml_diff>
--- a/data/mapmaker.xlsx
+++ b/data/mapmaker.xlsx
@@ -6180,7 +6180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F794"/>
+  <dimension ref="A1:F793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20171,17 +20171,25 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="C583" t="inlineStr"/>
+          <t>ERA5</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>ERA5-BO-0001</t>
+        </is>
+      </c>
       <c r="D583" t="n">
-        <v>3.15</v>
+        <v>1.625</v>
       </c>
       <c r="E583" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="F583" t="inlineStr"/>
+        <v>50.125</v>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>ERA5-BO-0001</t>
+        </is>
+      </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -20196,20 +20204,16 @@
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>ERA5-BO-0001</t>
+          <t>ERA5-BO-0002</t>
         </is>
       </c>
       <c r="D584" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E584" t="n">
         <v>50.125</v>
       </c>
-      <c r="F584" t="inlineStr">
-        <is>
-          <t>ERA5-BO-0001</t>
-        </is>
-      </c>
+      <c r="F584" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -20224,11 +20228,11 @@
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>ERA5-BO-0002</t>
+          <t>ERA5-BO-0003</t>
         </is>
       </c>
       <c r="D585" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E585" t="n">
         <v>50.125</v>
@@ -20248,11 +20252,11 @@
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>ERA5-BO-0003</t>
+          <t>ERA5-BO-0004</t>
         </is>
       </c>
       <c r="D586" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E586" t="n">
         <v>50.125</v>
@@ -20272,11 +20276,11 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>ERA5-BO-0004</t>
+          <t>ERA5-BO-0005</t>
         </is>
       </c>
       <c r="D587" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E587" t="n">
         <v>50.125</v>
@@ -20296,11 +20300,11 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>ERA5-BO-0005</t>
+          <t>ERA5-BO-0006</t>
         </is>
       </c>
       <c r="D588" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E588" t="n">
         <v>50.125</v>
@@ -20320,11 +20324,11 @@
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>ERA5-BO-0006</t>
+          <t>ERA5-BO-0007</t>
         </is>
       </c>
       <c r="D589" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E589" t="n">
         <v>50.125</v>
@@ -20344,11 +20348,11 @@
       </c>
       <c r="C590" t="inlineStr">
         <is>
-          <t>ERA5-BO-0007</t>
+          <t>ERA5-BO-0008</t>
         </is>
       </c>
       <c r="D590" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E590" t="n">
         <v>50.125</v>
@@ -20368,11 +20372,11 @@
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>ERA5-BO-0008</t>
+          <t>ERA5-BO-0009</t>
         </is>
       </c>
       <c r="D591" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E591" t="n">
         <v>50.125</v>
@@ -20392,11 +20396,11 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>ERA5-BO-0009</t>
+          <t>ERA5-BO-0010</t>
         </is>
       </c>
       <c r="D592" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E592" t="n">
         <v>50.125</v>
@@ -20416,11 +20420,11 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ERA5-BO-0010</t>
+          <t>ERA5-BO-0011</t>
         </is>
       </c>
       <c r="D593" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E593" t="n">
         <v>50.125</v>
@@ -20440,11 +20444,11 @@
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>ERA5-BO-0011</t>
+          <t>ERA5-BO-0012</t>
         </is>
       </c>
       <c r="D594" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E594" t="n">
         <v>50.125</v>
@@ -20464,11 +20468,11 @@
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>ERA5-BO-0012</t>
+          <t>ERA5-BO-0013</t>
         </is>
       </c>
       <c r="D595" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E595" t="n">
         <v>50.125</v>
@@ -20488,14 +20492,14 @@
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>ERA5-BO-0013</t>
+          <t>ERA5-BO-0014</t>
         </is>
       </c>
       <c r="D596" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E596" t="n">
-        <v>50.125</v>
+        <v>50.375</v>
       </c>
       <c r="F596" t="inlineStr"/>
     </row>
@@ -20512,11 +20516,11 @@
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>ERA5-BO-0014</t>
+          <t>ERA5-BO-0015</t>
         </is>
       </c>
       <c r="D597" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E597" t="n">
         <v>50.375</v>
@@ -20536,11 +20540,11 @@
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>ERA5-BO-0015</t>
+          <t>ERA5-BO-0016</t>
         </is>
       </c>
       <c r="D598" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E598" t="n">
         <v>50.375</v>
@@ -20560,11 +20564,11 @@
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>ERA5-BO-0016</t>
+          <t>ERA5-BO-0017</t>
         </is>
       </c>
       <c r="D599" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E599" t="n">
         <v>50.375</v>
@@ -20584,11 +20588,11 @@
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>ERA5-BO-0017</t>
+          <t>ERA5-BO-0018</t>
         </is>
       </c>
       <c r="D600" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E600" t="n">
         <v>50.375</v>
@@ -20608,11 +20612,11 @@
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>ERA5-BO-0018</t>
+          <t>ERA5-BO-0019</t>
         </is>
       </c>
       <c r="D601" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E601" t="n">
         <v>50.375</v>
@@ -20632,11 +20636,11 @@
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>ERA5-BO-0019</t>
+          <t>ERA5-BO-0020</t>
         </is>
       </c>
       <c r="D602" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E602" t="n">
         <v>50.375</v>
@@ -20656,11 +20660,11 @@
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>ERA5-BO-0020</t>
+          <t>ERA5-BO-0021</t>
         </is>
       </c>
       <c r="D603" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E603" t="n">
         <v>50.375</v>
@@ -20680,11 +20684,11 @@
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>ERA5-BO-0021</t>
+          <t>ERA5-BO-0022</t>
         </is>
       </c>
       <c r="D604" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E604" t="n">
         <v>50.375</v>
@@ -20704,11 +20708,11 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>ERA5-BO-0022</t>
+          <t>ERA5-BO-0023</t>
         </is>
       </c>
       <c r="D605" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E605" t="n">
         <v>50.375</v>
@@ -20728,11 +20732,11 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>ERA5-BO-0023</t>
+          <t>ERA5-BO-0024</t>
         </is>
       </c>
       <c r="D606" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E606" t="n">
         <v>50.375</v>
@@ -20752,11 +20756,11 @@
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>ERA5-BO-0024</t>
+          <t>ERA5-BO-0025</t>
         </is>
       </c>
       <c r="D607" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E607" t="n">
         <v>50.375</v>
@@ -20776,11 +20780,11 @@
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>ERA5-BO-0025</t>
+          <t>ERA5-BO-0026</t>
         </is>
       </c>
       <c r="D608" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E608" t="n">
         <v>50.375</v>
@@ -20800,14 +20804,14 @@
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>ERA5-BO-0026</t>
+          <t>ERA5-BO-0027</t>
         </is>
       </c>
       <c r="D609" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E609" t="n">
-        <v>50.375</v>
+        <v>50.625</v>
       </c>
       <c r="F609" t="inlineStr"/>
     </row>
@@ -20824,11 +20828,11 @@
       </c>
       <c r="C610" t="inlineStr">
         <is>
-          <t>ERA5-BO-0027</t>
+          <t>ERA5-BO-0028</t>
         </is>
       </c>
       <c r="D610" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E610" t="n">
         <v>50.625</v>
@@ -20848,11 +20852,11 @@
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>ERA5-BO-0028</t>
+          <t>ERA5-BO-0029</t>
         </is>
       </c>
       <c r="D611" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E611" t="n">
         <v>50.625</v>
@@ -20872,11 +20876,11 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>ERA5-BO-0029</t>
+          <t>ERA5-BO-0030</t>
         </is>
       </c>
       <c r="D612" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E612" t="n">
         <v>50.625</v>
@@ -20896,11 +20900,11 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>ERA5-BO-0030</t>
+          <t>ERA5-BO-0031</t>
         </is>
       </c>
       <c r="D613" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E613" t="n">
         <v>50.625</v>
@@ -20920,11 +20924,11 @@
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>ERA5-BO-0031</t>
+          <t>ERA5-BO-0032</t>
         </is>
       </c>
       <c r="D614" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E614" t="n">
         <v>50.625</v>
@@ -20944,11 +20948,11 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>ERA5-BO-0032</t>
+          <t>ERA5-BO-0033</t>
         </is>
       </c>
       <c r="D615" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E615" t="n">
         <v>50.625</v>
@@ -20968,11 +20972,11 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>ERA5-BO-0033</t>
+          <t>ERA5-BO-0034</t>
         </is>
       </c>
       <c r="D616" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E616" t="n">
         <v>50.625</v>
@@ -20992,11 +20996,11 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>ERA5-BO-0034</t>
+          <t>ERA5-BO-0035</t>
         </is>
       </c>
       <c r="D617" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E617" t="n">
         <v>50.625</v>
@@ -21016,11 +21020,11 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>ERA5-BO-0035</t>
+          <t>ERA5-BO-0036</t>
         </is>
       </c>
       <c r="D618" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E618" t="n">
         <v>50.625</v>
@@ -21040,11 +21044,11 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>ERA5-BO-0036</t>
+          <t>ERA5-BO-0037</t>
         </is>
       </c>
       <c r="D619" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E619" t="n">
         <v>50.625</v>
@@ -21064,11 +21068,11 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>ERA5-BO-0037</t>
+          <t>ERA5-BO-0038</t>
         </is>
       </c>
       <c r="D620" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E620" t="n">
         <v>50.625</v>
@@ -21088,11 +21092,11 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>ERA5-BO-0038</t>
+          <t>ERA5-BO-0039</t>
         </is>
       </c>
       <c r="D621" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E621" t="n">
         <v>50.625</v>
@@ -21112,14 +21116,14 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>ERA5-BO-0039</t>
+          <t>ERA5-BO-0040</t>
         </is>
       </c>
       <c r="D622" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E622" t="n">
-        <v>50.625</v>
+        <v>50.875</v>
       </c>
       <c r="F622" t="inlineStr"/>
     </row>
@@ -21136,11 +21140,11 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>ERA5-BO-0040</t>
+          <t>ERA5-BO-0041</t>
         </is>
       </c>
       <c r="D623" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E623" t="n">
         <v>50.875</v>
@@ -21160,11 +21164,11 @@
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>ERA5-BO-0041</t>
+          <t>ERA5-BO-0042</t>
         </is>
       </c>
       <c r="D624" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E624" t="n">
         <v>50.875</v>
@@ -21184,11 +21188,11 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>ERA5-BO-0042</t>
+          <t>ERA5-BO-0043</t>
         </is>
       </c>
       <c r="D625" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E625" t="n">
         <v>50.875</v>
@@ -21208,11 +21212,11 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>ERA5-BO-0043</t>
+          <t>ERA5-BO-0044</t>
         </is>
       </c>
       <c r="D626" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E626" t="n">
         <v>50.875</v>
@@ -21232,11 +21236,11 @@
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>ERA5-BO-0044</t>
+          <t>ERA5-BO-0045</t>
         </is>
       </c>
       <c r="D627" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E627" t="n">
         <v>50.875</v>
@@ -21256,11 +21260,11 @@
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>ERA5-BO-0045</t>
+          <t>ERA5-BO-0046</t>
         </is>
       </c>
       <c r="D628" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E628" t="n">
         <v>50.875</v>
@@ -21280,11 +21284,11 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>ERA5-BO-0046</t>
+          <t>ERA5-BO-0047</t>
         </is>
       </c>
       <c r="D629" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E629" t="n">
         <v>50.875</v>
@@ -21304,11 +21308,11 @@
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>ERA5-BO-0047</t>
+          <t>ERA5-BO-0048</t>
         </is>
       </c>
       <c r="D630" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E630" t="n">
         <v>50.875</v>
@@ -21328,11 +21332,11 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>ERA5-BO-0048</t>
+          <t>ERA5-BO-0049</t>
         </is>
       </c>
       <c r="D631" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E631" t="n">
         <v>50.875</v>
@@ -21352,11 +21356,11 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>ERA5-BO-0049</t>
+          <t>ERA5-BO-0050</t>
         </is>
       </c>
       <c r="D632" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E632" t="n">
         <v>50.875</v>
@@ -21376,11 +21380,11 @@
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>ERA5-BO-0050</t>
+          <t>ERA5-BO-0051</t>
         </is>
       </c>
       <c r="D633" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E633" t="n">
         <v>50.875</v>
@@ -21400,11 +21404,11 @@
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>ERA5-BO-0051</t>
+          <t>ERA5-BO-0052</t>
         </is>
       </c>
       <c r="D634" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E634" t="n">
         <v>50.875</v>
@@ -21424,14 +21428,14 @@
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>ERA5-BO-0052</t>
+          <t>ERA5-BO-0053</t>
         </is>
       </c>
       <c r="D635" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E635" t="n">
-        <v>50.875</v>
+        <v>51.125</v>
       </c>
       <c r="F635" t="inlineStr"/>
     </row>
@@ -21448,11 +21452,11 @@
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>ERA5-BO-0053</t>
+          <t>ERA5-BO-0054</t>
         </is>
       </c>
       <c r="D636" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E636" t="n">
         <v>51.125</v>
@@ -21472,11 +21476,11 @@
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>ERA5-BO-0054</t>
+          <t>ERA5-BO-0055</t>
         </is>
       </c>
       <c r="D637" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E637" t="n">
         <v>51.125</v>
@@ -21496,11 +21500,11 @@
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>ERA5-BO-0055</t>
+          <t>ERA5-BO-0056</t>
         </is>
       </c>
       <c r="D638" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E638" t="n">
         <v>51.125</v>
@@ -21520,11 +21524,11 @@
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>ERA5-BO-0056</t>
+          <t>ERA5-BO-0057</t>
         </is>
       </c>
       <c r="D639" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E639" t="n">
         <v>51.125</v>
@@ -21544,11 +21548,11 @@
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>ERA5-BO-0057</t>
+          <t>ERA5-BO-0058</t>
         </is>
       </c>
       <c r="D640" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E640" t="n">
         <v>51.125</v>
@@ -21568,11 +21572,11 @@
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>ERA5-BO-0058</t>
+          <t>ERA5-BO-0059</t>
         </is>
       </c>
       <c r="D641" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E641" t="n">
         <v>51.125</v>
@@ -21592,11 +21596,11 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>ERA5-BO-0059</t>
+          <t>ERA5-BO-0060</t>
         </is>
       </c>
       <c r="D642" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E642" t="n">
         <v>51.125</v>
@@ -21616,11 +21620,11 @@
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>ERA5-BO-0060</t>
+          <t>ERA5-BO-0061</t>
         </is>
       </c>
       <c r="D643" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E643" t="n">
         <v>51.125</v>
@@ -21640,11 +21644,11 @@
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>ERA5-BO-0061</t>
+          <t>ERA5-BO-0062</t>
         </is>
       </c>
       <c r="D644" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E644" t="n">
         <v>51.125</v>
@@ -21664,11 +21668,11 @@
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>ERA5-BO-0062</t>
+          <t>ERA5-BO-0063</t>
         </is>
       </c>
       <c r="D645" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E645" t="n">
         <v>51.125</v>
@@ -21688,11 +21692,11 @@
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>ERA5-BO-0063</t>
+          <t>ERA5-BO-0064</t>
         </is>
       </c>
       <c r="D646" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E646" t="n">
         <v>51.125</v>
@@ -21712,11 +21716,11 @@
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>ERA5-BO-0064</t>
+          <t>ERA5-BO-0065</t>
         </is>
       </c>
       <c r="D647" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E647" t="n">
         <v>51.125</v>
@@ -21736,14 +21740,14 @@
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>ERA5-BO-0065</t>
+          <t>ERA5-BO-0066</t>
         </is>
       </c>
       <c r="D648" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E648" t="n">
-        <v>51.125</v>
+        <v>51.375</v>
       </c>
       <c r="F648" t="inlineStr"/>
     </row>
@@ -21760,11 +21764,11 @@
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>ERA5-BO-0066</t>
+          <t>ERA5-BO-0067</t>
         </is>
       </c>
       <c r="D649" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E649" t="n">
         <v>51.375</v>
@@ -21784,11 +21788,11 @@
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>ERA5-BO-0067</t>
+          <t>ERA5-BO-0068</t>
         </is>
       </c>
       <c r="D650" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E650" t="n">
         <v>51.375</v>
@@ -21808,11 +21812,11 @@
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>ERA5-BO-0068</t>
+          <t>ERA5-BO-0069</t>
         </is>
       </c>
       <c r="D651" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E651" t="n">
         <v>51.375</v>
@@ -21832,11 +21836,11 @@
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>ERA5-BO-0069</t>
+          <t>ERA5-BO-0070</t>
         </is>
       </c>
       <c r="D652" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E652" t="n">
         <v>51.375</v>
@@ -21856,11 +21860,11 @@
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>ERA5-BO-0070</t>
+          <t>ERA5-BO-0071</t>
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E653" t="n">
         <v>51.375</v>
@@ -21880,11 +21884,11 @@
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>ERA5-BO-0071</t>
+          <t>ERA5-BO-0072</t>
         </is>
       </c>
       <c r="D654" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E654" t="n">
         <v>51.375</v>
@@ -21904,11 +21908,11 @@
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>ERA5-BO-0072</t>
+          <t>ERA5-BO-0073</t>
         </is>
       </c>
       <c r="D655" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E655" t="n">
         <v>51.375</v>
@@ -21928,11 +21932,11 @@
       </c>
       <c r="C656" t="inlineStr">
         <is>
-          <t>ERA5-BO-0073</t>
+          <t>ERA5-BO-0074</t>
         </is>
       </c>
       <c r="D656" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E656" t="n">
         <v>51.375</v>
@@ -21952,11 +21956,11 @@
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>ERA5-BO-0074</t>
+          <t>ERA5-BO-0075</t>
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E657" t="n">
         <v>51.375</v>
@@ -21976,11 +21980,11 @@
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>ERA5-BO-0075</t>
+          <t>ERA5-BO-0076</t>
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E658" t="n">
         <v>51.375</v>
@@ -22000,11 +22004,11 @@
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>ERA5-BO-0076</t>
+          <t>ERA5-BO-0077</t>
         </is>
       </c>
       <c r="D659" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E659" t="n">
         <v>51.375</v>
@@ -22024,11 +22028,11 @@
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>ERA5-BO-0077</t>
+          <t>ERA5-BO-0078</t>
         </is>
       </c>
       <c r="D660" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E660" t="n">
         <v>51.375</v>
@@ -22048,14 +22052,14 @@
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>ERA5-BO-0078</t>
+          <t>ERA5-BO-0079</t>
         </is>
       </c>
       <c r="D661" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E661" t="n">
-        <v>51.375</v>
+        <v>51.625</v>
       </c>
       <c r="F661" t="inlineStr"/>
     </row>
@@ -22072,11 +22076,11 @@
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>ERA5-BO-0079</t>
+          <t>ERA5-BO-0080</t>
         </is>
       </c>
       <c r="D662" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E662" t="n">
         <v>51.625</v>
@@ -22096,11 +22100,11 @@
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>ERA5-BO-0080</t>
+          <t>ERA5-BO-0081</t>
         </is>
       </c>
       <c r="D663" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E663" t="n">
         <v>51.625</v>
@@ -22120,11 +22124,11 @@
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>ERA5-BO-0081</t>
+          <t>ERA5-BO-0082</t>
         </is>
       </c>
       <c r="D664" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E664" t="n">
         <v>51.625</v>
@@ -22144,11 +22148,11 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>ERA5-BO-0082</t>
+          <t>ERA5-BO-0083</t>
         </is>
       </c>
       <c r="D665" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E665" t="n">
         <v>51.625</v>
@@ -22168,11 +22172,11 @@
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>ERA5-BO-0083</t>
+          <t>ERA5-BO-0084</t>
         </is>
       </c>
       <c r="D666" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E666" t="n">
         <v>51.625</v>
@@ -22192,11 +22196,11 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>ERA5-BO-0084</t>
+          <t>ERA5-BO-0085</t>
         </is>
       </c>
       <c r="D667" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E667" t="n">
         <v>51.625</v>
@@ -22216,11 +22220,11 @@
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>ERA5-BO-0085</t>
+          <t>ERA5-BO-0086</t>
         </is>
       </c>
       <c r="D668" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E668" t="n">
         <v>51.625</v>
@@ -22240,11 +22244,11 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>ERA5-BO-0086</t>
+          <t>ERA5-BO-0087</t>
         </is>
       </c>
       <c r="D669" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E669" t="n">
         <v>51.625</v>
@@ -22264,11 +22268,11 @@
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>ERA5-BO-0087</t>
+          <t>ERA5-BO-0088</t>
         </is>
       </c>
       <c r="D670" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E670" t="n">
         <v>51.625</v>
@@ -22288,11 +22292,11 @@
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>ERA5-BO-0088</t>
+          <t>ERA5-BO-0089</t>
         </is>
       </c>
       <c r="D671" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E671" t="n">
         <v>51.625</v>
@@ -22312,11 +22316,11 @@
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>ERA5-BO-0089</t>
+          <t>ERA5-BO-0090</t>
         </is>
       </c>
       <c r="D672" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E672" t="n">
         <v>51.625</v>
@@ -22336,11 +22340,11 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>ERA5-BO-0090</t>
+          <t>ERA5-BO-0091</t>
         </is>
       </c>
       <c r="D673" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E673" t="n">
         <v>51.625</v>
@@ -22360,14 +22364,14 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>ERA5-BO-0091</t>
+          <t>ERA5-BO-0092</t>
         </is>
       </c>
       <c r="D674" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E674" t="n">
-        <v>51.625</v>
+        <v>51.875</v>
       </c>
       <c r="F674" t="inlineStr"/>
     </row>
@@ -22384,11 +22388,11 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>ERA5-BO-0092</t>
+          <t>ERA5-BO-0093</t>
         </is>
       </c>
       <c r="D675" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E675" t="n">
         <v>51.875</v>
@@ -22408,11 +22412,11 @@
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>ERA5-BO-0093</t>
+          <t>ERA5-BO-0094</t>
         </is>
       </c>
       <c r="D676" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E676" t="n">
         <v>51.875</v>
@@ -22432,11 +22436,11 @@
       </c>
       <c r="C677" t="inlineStr">
         <is>
-          <t>ERA5-BO-0094</t>
+          <t>ERA5-BO-0095</t>
         </is>
       </c>
       <c r="D677" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E677" t="n">
         <v>51.875</v>
@@ -22456,11 +22460,11 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>ERA5-BO-0095</t>
+          <t>ERA5-BO-0096</t>
         </is>
       </c>
       <c r="D678" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E678" t="n">
         <v>51.875</v>
@@ -22480,11 +22484,11 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>ERA5-BO-0096</t>
+          <t>ERA5-BO-0097</t>
         </is>
       </c>
       <c r="D679" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E679" t="n">
         <v>51.875</v>
@@ -22504,11 +22508,11 @@
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>ERA5-BO-0097</t>
+          <t>ERA5-BO-0098</t>
         </is>
       </c>
       <c r="D680" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E680" t="n">
         <v>51.875</v>
@@ -22528,11 +22532,11 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>ERA5-BO-0098</t>
+          <t>ERA5-BO-0099</t>
         </is>
       </c>
       <c r="D681" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E681" t="n">
         <v>51.875</v>
@@ -22552,11 +22556,11 @@
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>ERA5-BO-0099</t>
+          <t>ERA5-BO-0100</t>
         </is>
       </c>
       <c r="D682" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E682" t="n">
         <v>51.875</v>
@@ -22576,11 +22580,11 @@
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>ERA5-BO-0100</t>
+          <t>ERA5-BO-0101</t>
         </is>
       </c>
       <c r="D683" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E683" t="n">
         <v>51.875</v>
@@ -22600,11 +22604,11 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>ERA5-BO-0101</t>
+          <t>ERA5-BO-0102</t>
         </is>
       </c>
       <c r="D684" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E684" t="n">
         <v>51.875</v>
@@ -22624,11 +22628,11 @@
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>ERA5-BO-0102</t>
+          <t>ERA5-BO-0103</t>
         </is>
       </c>
       <c r="D685" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E685" t="n">
         <v>51.875</v>
@@ -22648,11 +22652,11 @@
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>ERA5-BO-0103</t>
+          <t>ERA5-BO-0104</t>
         </is>
       </c>
       <c r="D686" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E686" t="n">
         <v>51.875</v>
@@ -22672,14 +22676,14 @@
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>ERA5-BO-0104</t>
+          <t>ERA5-BO-0105</t>
         </is>
       </c>
       <c r="D687" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E687" t="n">
-        <v>51.875</v>
+        <v>52.125</v>
       </c>
       <c r="F687" t="inlineStr"/>
     </row>
@@ -22696,11 +22700,11 @@
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>ERA5-BO-0105</t>
+          <t>ERA5-BO-0106</t>
         </is>
       </c>
       <c r="D688" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E688" t="n">
         <v>52.125</v>
@@ -22720,11 +22724,11 @@
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>ERA5-BO-0106</t>
+          <t>ERA5-BO-0107</t>
         </is>
       </c>
       <c r="D689" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E689" t="n">
         <v>52.125</v>
@@ -22744,11 +22748,11 @@
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>ERA5-BO-0107</t>
+          <t>ERA5-BO-0108</t>
         </is>
       </c>
       <c r="D690" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E690" t="n">
         <v>52.125</v>
@@ -22768,11 +22772,11 @@
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>ERA5-BO-0108</t>
+          <t>ERA5-BO-0109</t>
         </is>
       </c>
       <c r="D691" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E691" t="n">
         <v>52.125</v>
@@ -22792,11 +22796,11 @@
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>ERA5-BO-0109</t>
+          <t>ERA5-BO-0110</t>
         </is>
       </c>
       <c r="D692" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E692" t="n">
         <v>52.125</v>
@@ -22816,11 +22820,11 @@
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>ERA5-BO-0110</t>
+          <t>ERA5-BO-0111</t>
         </is>
       </c>
       <c r="D693" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E693" t="n">
         <v>52.125</v>
@@ -22840,11 +22844,11 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>ERA5-BO-0111</t>
+          <t>ERA5-BO-0112</t>
         </is>
       </c>
       <c r="D694" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E694" t="n">
         <v>52.125</v>
@@ -22864,11 +22868,11 @@
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>ERA5-BO-0112</t>
+          <t>ERA5-BO-0113</t>
         </is>
       </c>
       <c r="D695" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E695" t="n">
         <v>52.125</v>
@@ -22888,11 +22892,11 @@
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>ERA5-BO-0113</t>
+          <t>ERA5-BO-0114</t>
         </is>
       </c>
       <c r="D696" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E696" t="n">
         <v>52.125</v>
@@ -22912,11 +22916,11 @@
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>ERA5-BO-0114</t>
+          <t>ERA5-BO-0115</t>
         </is>
       </c>
       <c r="D697" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E697" t="n">
         <v>52.125</v>
@@ -22936,11 +22940,11 @@
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>ERA5-BO-0115</t>
+          <t>ERA5-BO-0116</t>
         </is>
       </c>
       <c r="D698" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E698" t="n">
         <v>52.125</v>
@@ -22960,11 +22964,11 @@
       </c>
       <c r="C699" t="inlineStr">
         <is>
-          <t>ERA5-BO-0116</t>
+          <t>ERA5-BO-0117</t>
         </is>
       </c>
       <c r="D699" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E699" t="n">
         <v>52.125</v>
@@ -22984,14 +22988,14 @@
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>ERA5-BO-0117</t>
+          <t>ERA5-BO-0118</t>
         </is>
       </c>
       <c r="D700" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E700" t="n">
-        <v>52.125</v>
+        <v>52.375</v>
       </c>
       <c r="F700" t="inlineStr"/>
     </row>
@@ -23008,11 +23012,11 @@
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>ERA5-BO-0118</t>
+          <t>ERA5-BO-0119</t>
         </is>
       </c>
       <c r="D701" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E701" t="n">
         <v>52.375</v>
@@ -23032,11 +23036,11 @@
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>ERA5-BO-0119</t>
+          <t>ERA5-BO-0120</t>
         </is>
       </c>
       <c r="D702" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E702" t="n">
         <v>52.375</v>
@@ -23056,11 +23060,11 @@
       </c>
       <c r="C703" t="inlineStr">
         <is>
-          <t>ERA5-BO-0120</t>
+          <t>ERA5-BO-0121</t>
         </is>
       </c>
       <c r="D703" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E703" t="n">
         <v>52.375</v>
@@ -23080,11 +23084,11 @@
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>ERA5-BO-0121</t>
+          <t>ERA5-BO-0122</t>
         </is>
       </c>
       <c r="D704" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E704" t="n">
         <v>52.375</v>
@@ -23104,11 +23108,11 @@
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>ERA5-BO-0122</t>
+          <t>ERA5-BO-0123</t>
         </is>
       </c>
       <c r="D705" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E705" t="n">
         <v>52.375</v>
@@ -23128,11 +23132,11 @@
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>ERA5-BO-0123</t>
+          <t>ERA5-BO-0124</t>
         </is>
       </c>
       <c r="D706" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E706" t="n">
         <v>52.375</v>
@@ -23152,11 +23156,11 @@
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>ERA5-BO-0124</t>
+          <t>ERA5-BO-0125</t>
         </is>
       </c>
       <c r="D707" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E707" t="n">
         <v>52.375</v>
@@ -23176,11 +23180,11 @@
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>ERA5-BO-0125</t>
+          <t>ERA5-BO-0126</t>
         </is>
       </c>
       <c r="D708" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E708" t="n">
         <v>52.375</v>
@@ -23200,11 +23204,11 @@
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>ERA5-BO-0126</t>
+          <t>ERA5-BO-0127</t>
         </is>
       </c>
       <c r="D709" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E709" t="n">
         <v>52.375</v>
@@ -23224,11 +23228,11 @@
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>ERA5-BO-0127</t>
+          <t>ERA5-BO-0128</t>
         </is>
       </c>
       <c r="D710" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E710" t="n">
         <v>52.375</v>
@@ -23248,11 +23252,11 @@
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>ERA5-BO-0128</t>
+          <t>ERA5-BO-0129</t>
         </is>
       </c>
       <c r="D711" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E711" t="n">
         <v>52.375</v>
@@ -23272,11 +23276,11 @@
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>ERA5-BO-0129</t>
+          <t>ERA5-BO-0130</t>
         </is>
       </c>
       <c r="D712" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E712" t="n">
         <v>52.375</v>
@@ -23296,14 +23300,14 @@
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>ERA5-BO-0130</t>
+          <t>ERA5-BO-0131</t>
         </is>
       </c>
       <c r="D713" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E713" t="n">
-        <v>52.375</v>
+        <v>52.625</v>
       </c>
       <c r="F713" t="inlineStr"/>
     </row>
@@ -23320,11 +23324,11 @@
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>ERA5-BO-0131</t>
+          <t>ERA5-BO-0132</t>
         </is>
       </c>
       <c r="D714" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E714" t="n">
         <v>52.625</v>
@@ -23344,11 +23348,11 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>ERA5-BO-0132</t>
+          <t>ERA5-BO-0133</t>
         </is>
       </c>
       <c r="D715" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E715" t="n">
         <v>52.625</v>
@@ -23368,11 +23372,11 @@
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>ERA5-BO-0133</t>
+          <t>ERA5-BO-0134</t>
         </is>
       </c>
       <c r="D716" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E716" t="n">
         <v>52.625</v>
@@ -23392,11 +23396,11 @@
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>ERA5-BO-0134</t>
+          <t>ERA5-BO-0135</t>
         </is>
       </c>
       <c r="D717" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E717" t="n">
         <v>52.625</v>
@@ -23416,11 +23420,11 @@
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>ERA5-BO-0135</t>
+          <t>ERA5-BO-0136</t>
         </is>
       </c>
       <c r="D718" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E718" t="n">
         <v>52.625</v>
@@ -23440,11 +23444,11 @@
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>ERA5-BO-0136</t>
+          <t>ERA5-BO-0137</t>
         </is>
       </c>
       <c r="D719" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E719" t="n">
         <v>52.625</v>
@@ -23464,11 +23468,11 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>ERA5-BO-0137</t>
+          <t>ERA5-BO-0138</t>
         </is>
       </c>
       <c r="D720" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E720" t="n">
         <v>52.625</v>
@@ -23488,11 +23492,11 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>ERA5-BO-0138</t>
+          <t>ERA5-BO-0139</t>
         </is>
       </c>
       <c r="D721" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E721" t="n">
         <v>52.625</v>
@@ -23512,11 +23516,11 @@
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>ERA5-BO-0139</t>
+          <t>ERA5-BO-0140</t>
         </is>
       </c>
       <c r="D722" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E722" t="n">
         <v>52.625</v>
@@ -23536,11 +23540,11 @@
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>ERA5-BO-0140</t>
+          <t>ERA5-BO-0141</t>
         </is>
       </c>
       <c r="D723" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E723" t="n">
         <v>52.625</v>
@@ -23560,11 +23564,11 @@
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>ERA5-BO-0141</t>
+          <t>ERA5-BO-0142</t>
         </is>
       </c>
       <c r="D724" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E724" t="n">
         <v>52.625</v>
@@ -23584,11 +23588,11 @@
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>ERA5-BO-0142</t>
+          <t>ERA5-BO-0143</t>
         </is>
       </c>
       <c r="D725" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E725" t="n">
         <v>52.625</v>
@@ -23608,14 +23612,14 @@
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>ERA5-BO-0143</t>
+          <t>ERA5-BO-0144</t>
         </is>
       </c>
       <c r="D726" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E726" t="n">
-        <v>52.625</v>
+        <v>52.875</v>
       </c>
       <c r="F726" t="inlineStr"/>
     </row>
@@ -23632,11 +23636,11 @@
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>ERA5-BO-0144</t>
+          <t>ERA5-BO-0145</t>
         </is>
       </c>
       <c r="D727" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E727" t="n">
         <v>52.875</v>
@@ -23656,11 +23660,11 @@
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>ERA5-BO-0145</t>
+          <t>ERA5-BO-0146</t>
         </is>
       </c>
       <c r="D728" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E728" t="n">
         <v>52.875</v>
@@ -23680,11 +23684,11 @@
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>ERA5-BO-0146</t>
+          <t>ERA5-BO-0147</t>
         </is>
       </c>
       <c r="D729" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E729" t="n">
         <v>52.875</v>
@@ -23704,11 +23708,11 @@
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>ERA5-BO-0147</t>
+          <t>ERA5-BO-0148</t>
         </is>
       </c>
       <c r="D730" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E730" t="n">
         <v>52.875</v>
@@ -23728,11 +23732,11 @@
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>ERA5-BO-0148</t>
+          <t>ERA5-BO-0149</t>
         </is>
       </c>
       <c r="D731" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E731" t="n">
         <v>52.875</v>
@@ -23752,11 +23756,11 @@
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>ERA5-BO-0149</t>
+          <t>ERA5-BO-0150</t>
         </is>
       </c>
       <c r="D732" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E732" t="n">
         <v>52.875</v>
@@ -23776,11 +23780,11 @@
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>ERA5-BO-0150</t>
+          <t>ERA5-BO-0151</t>
         </is>
       </c>
       <c r="D733" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E733" t="n">
         <v>52.875</v>
@@ -23800,11 +23804,11 @@
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>ERA5-BO-0151</t>
+          <t>ERA5-BO-0152</t>
         </is>
       </c>
       <c r="D734" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E734" t="n">
         <v>52.875</v>
@@ -23824,11 +23828,11 @@
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>ERA5-BO-0152</t>
+          <t>ERA5-BO-0153</t>
         </is>
       </c>
       <c r="D735" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E735" t="n">
         <v>52.875</v>
@@ -23848,11 +23852,11 @@
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>ERA5-BO-0153</t>
+          <t>ERA5-BO-0154</t>
         </is>
       </c>
       <c r="D736" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E736" t="n">
         <v>52.875</v>
@@ -23872,11 +23876,11 @@
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>ERA5-BO-0154</t>
+          <t>ERA5-BO-0155</t>
         </is>
       </c>
       <c r="D737" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E737" t="n">
         <v>52.875</v>
@@ -23896,11 +23900,11 @@
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>ERA5-BO-0155</t>
+          <t>ERA5-BO-0156</t>
         </is>
       </c>
       <c r="D738" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E738" t="n">
         <v>52.875</v>
@@ -23920,14 +23924,14 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>ERA5-BO-0156</t>
+          <t>ERA5-BO-0157</t>
         </is>
       </c>
       <c r="D739" t="n">
-        <v>4.625</v>
+        <v>1.625</v>
       </c>
       <c r="E739" t="n">
-        <v>52.875</v>
+        <v>53.125</v>
       </c>
       <c r="F739" t="inlineStr"/>
     </row>
@@ -23944,11 +23948,11 @@
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>ERA5-BO-0157</t>
+          <t>ERA5-BO-0158</t>
         </is>
       </c>
       <c r="D740" t="n">
-        <v>1.625</v>
+        <v>1.875</v>
       </c>
       <c r="E740" t="n">
         <v>53.125</v>
@@ -23968,11 +23972,11 @@
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>ERA5-BO-0158</t>
+          <t>ERA5-BO-0159</t>
         </is>
       </c>
       <c r="D741" t="n">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="E741" t="n">
         <v>53.125</v>
@@ -23992,11 +23996,11 @@
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>ERA5-BO-0159</t>
+          <t>ERA5-BO-0160</t>
         </is>
       </c>
       <c r="D742" t="n">
-        <v>2.125</v>
+        <v>2.375</v>
       </c>
       <c r="E742" t="n">
         <v>53.125</v>
@@ -24016,11 +24020,11 @@
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>ERA5-BO-0160</t>
+          <t>ERA5-BO-0161</t>
         </is>
       </c>
       <c r="D743" t="n">
-        <v>2.375</v>
+        <v>2.625</v>
       </c>
       <c r="E743" t="n">
         <v>53.125</v>
@@ -24040,11 +24044,11 @@
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>ERA5-BO-0161</t>
+          <t>ERA5-BO-0162</t>
         </is>
       </c>
       <c r="D744" t="n">
-        <v>2.625</v>
+        <v>2.875</v>
       </c>
       <c r="E744" t="n">
         <v>53.125</v>
@@ -24064,11 +24068,11 @@
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>ERA5-BO-0162</t>
+          <t>ERA5-BO-0163</t>
         </is>
       </c>
       <c r="D745" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
       <c r="E745" t="n">
         <v>53.125</v>
@@ -24088,11 +24092,11 @@
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>ERA5-BO-0163</t>
+          <t>ERA5-BO-0164</t>
         </is>
       </c>
       <c r="D746" t="n">
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="E746" t="n">
         <v>53.125</v>
@@ -24112,11 +24116,11 @@
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>ERA5-BO-0164</t>
+          <t>ERA5-BO-0165</t>
         </is>
       </c>
       <c r="D747" t="n">
-        <v>3.375</v>
+        <v>3.625</v>
       </c>
       <c r="E747" t="n">
         <v>53.125</v>
@@ -24136,11 +24140,11 @@
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>ERA5-BO-0165</t>
+          <t>ERA5-BO-0166</t>
         </is>
       </c>
       <c r="D748" t="n">
-        <v>3.625</v>
+        <v>3.875</v>
       </c>
       <c r="E748" t="n">
         <v>53.125</v>
@@ -24160,11 +24164,11 @@
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>ERA5-BO-0166</t>
+          <t>ERA5-BO-0167</t>
         </is>
       </c>
       <c r="D749" t="n">
-        <v>3.875</v>
+        <v>4.125</v>
       </c>
       <c r="E749" t="n">
         <v>53.125</v>
@@ -24184,11 +24188,11 @@
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>ERA5-BO-0167</t>
+          <t>ERA5-BO-0168</t>
         </is>
       </c>
       <c r="D750" t="n">
-        <v>4.125</v>
+        <v>4.375</v>
       </c>
       <c r="E750" t="n">
         <v>53.125</v>
@@ -24208,11 +24212,11 @@
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>ERA5-BO-0168</t>
+          <t>ERA5-BO-0169</t>
         </is>
       </c>
       <c r="D751" t="n">
-        <v>4.375</v>
+        <v>4.625</v>
       </c>
       <c r="E751" t="n">
         <v>53.125</v>
@@ -24227,21 +24231,25 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>ERA5</t>
+          <t>MERRA2</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>ERA5-BO-0169</t>
+          <t>MERRA2-BO-0001</t>
         </is>
       </c>
       <c r="D752" t="n">
-        <v>4.625</v>
+        <v>1.5625</v>
       </c>
       <c r="E752" t="n">
-        <v>53.125</v>
-      </c>
-      <c r="F752" t="inlineStr"/>
+        <v>50.25</v>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>MERRA2-BO-0001</t>
+        </is>
+      </c>
     </row>
     <row r="753">
       <c r="A753" t="inlineStr">
@@ -24256,20 +24264,16 @@
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0001</t>
+          <t>MERRA2-BO-0002</t>
         </is>
       </c>
       <c r="D753" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E753" t="n">
         <v>50.25</v>
       </c>
-      <c r="F753" t="inlineStr">
-        <is>
-          <t>MERRA2-BO-0001</t>
-        </is>
-      </c>
+      <c r="F753" t="inlineStr"/>
     </row>
     <row r="754">
       <c r="A754" t="inlineStr">
@@ -24284,11 +24288,11 @@
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0002</t>
+          <t>MERRA2-BO-0003</t>
         </is>
       </c>
       <c r="D754" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E754" t="n">
         <v>50.25</v>
@@ -24308,11 +24312,11 @@
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0003</t>
+          <t>MERRA2-BO-0004</t>
         </is>
       </c>
       <c r="D755" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E755" t="n">
         <v>50.25</v>
@@ -24332,11 +24336,11 @@
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0004</t>
+          <t>MERRA2-BO-0005</t>
         </is>
       </c>
       <c r="D756" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E756" t="n">
         <v>50.25</v>
@@ -24356,11 +24360,11 @@
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0005</t>
+          <t>MERRA2-BO-0006</t>
         </is>
       </c>
       <c r="D757" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E757" t="n">
         <v>50.25</v>
@@ -24380,14 +24384,14 @@
       </c>
       <c r="C758" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0006</t>
+          <t>MERRA2-BO-0007</t>
         </is>
       </c>
       <c r="D758" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E758" t="n">
-        <v>50.25</v>
+        <v>50.75</v>
       </c>
       <c r="F758" t="inlineStr"/>
     </row>
@@ -24404,11 +24408,11 @@
       </c>
       <c r="C759" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0007</t>
+          <t>MERRA2-BO-0008</t>
         </is>
       </c>
       <c r="D759" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E759" t="n">
         <v>50.75</v>
@@ -24428,11 +24432,11 @@
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0008</t>
+          <t>MERRA2-BO-0009</t>
         </is>
       </c>
       <c r="D760" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E760" t="n">
         <v>50.75</v>
@@ -24452,11 +24456,11 @@
       </c>
       <c r="C761" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0009</t>
+          <t>MERRA2-BO-0010</t>
         </is>
       </c>
       <c r="D761" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E761" t="n">
         <v>50.75</v>
@@ -24476,11 +24480,11 @@
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0010</t>
+          <t>MERRA2-BO-0011</t>
         </is>
       </c>
       <c r="D762" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E762" t="n">
         <v>50.75</v>
@@ -24500,11 +24504,11 @@
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0011</t>
+          <t>MERRA2-BO-0012</t>
         </is>
       </c>
       <c r="D763" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E763" t="n">
         <v>50.75</v>
@@ -24524,14 +24528,14 @@
       </c>
       <c r="C764" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0012</t>
+          <t>MERRA2-BO-0013</t>
         </is>
       </c>
       <c r="D764" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E764" t="n">
-        <v>50.75</v>
+        <v>51.25</v>
       </c>
       <c r="F764" t="inlineStr"/>
     </row>
@@ -24548,11 +24552,11 @@
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0013</t>
+          <t>MERRA2-BO-0014</t>
         </is>
       </c>
       <c r="D765" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E765" t="n">
         <v>51.25</v>
@@ -24572,11 +24576,11 @@
       </c>
       <c r="C766" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0014</t>
+          <t>MERRA2-BO-0015</t>
         </is>
       </c>
       <c r="D766" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E766" t="n">
         <v>51.25</v>
@@ -24596,11 +24600,11 @@
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0015</t>
+          <t>MERRA2-BO-0016</t>
         </is>
       </c>
       <c r="D767" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E767" t="n">
         <v>51.25</v>
@@ -24620,11 +24624,11 @@
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0016</t>
+          <t>MERRA2-BO-0017</t>
         </is>
       </c>
       <c r="D768" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E768" t="n">
         <v>51.25</v>
@@ -24644,11 +24648,11 @@
       </c>
       <c r="C769" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0017</t>
+          <t>MERRA2-BO-0018</t>
         </is>
       </c>
       <c r="D769" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E769" t="n">
         <v>51.25</v>
@@ -24668,14 +24672,14 @@
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0018</t>
+          <t>MERRA2-BO-0019</t>
         </is>
       </c>
       <c r="D770" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E770" t="n">
-        <v>51.25</v>
+        <v>51.75</v>
       </c>
       <c r="F770" t="inlineStr"/>
     </row>
@@ -24692,11 +24696,11 @@
       </c>
       <c r="C771" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0019</t>
+          <t>MERRA2-BO-0020</t>
         </is>
       </c>
       <c r="D771" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E771" t="n">
         <v>51.75</v>
@@ -24716,11 +24720,11 @@
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0020</t>
+          <t>MERRA2-BO-0021</t>
         </is>
       </c>
       <c r="D772" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E772" t="n">
         <v>51.75</v>
@@ -24740,11 +24744,11 @@
       </c>
       <c r="C773" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0021</t>
+          <t>MERRA2-BO-0022</t>
         </is>
       </c>
       <c r="D773" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E773" t="n">
         <v>51.75</v>
@@ -24764,11 +24768,11 @@
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0022</t>
+          <t>MERRA2-BO-0023</t>
         </is>
       </c>
       <c r="D774" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E774" t="n">
         <v>51.75</v>
@@ -24788,11 +24792,11 @@
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0023</t>
+          <t>MERRA2-BO-0024</t>
         </is>
       </c>
       <c r="D775" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E775" t="n">
         <v>51.75</v>
@@ -24812,14 +24816,14 @@
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0024</t>
+          <t>MERRA2-BO-0025</t>
         </is>
       </c>
       <c r="D776" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E776" t="n">
-        <v>51.75</v>
+        <v>52.25</v>
       </c>
       <c r="F776" t="inlineStr"/>
     </row>
@@ -24836,11 +24840,11 @@
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0025</t>
+          <t>MERRA2-BO-0026</t>
         </is>
       </c>
       <c r="D777" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E777" t="n">
         <v>52.25</v>
@@ -24860,11 +24864,11 @@
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0026</t>
+          <t>MERRA2-BO-0027</t>
         </is>
       </c>
       <c r="D778" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E778" t="n">
         <v>52.25</v>
@@ -24884,11 +24888,11 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0027</t>
+          <t>MERRA2-BO-0028</t>
         </is>
       </c>
       <c r="D779" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E779" t="n">
         <v>52.25</v>
@@ -24908,11 +24912,11 @@
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0028</t>
+          <t>MERRA2-BO-0029</t>
         </is>
       </c>
       <c r="D780" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E780" t="n">
         <v>52.25</v>
@@ -24932,11 +24936,11 @@
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0029</t>
+          <t>MERRA2-BO-0030</t>
         </is>
       </c>
       <c r="D781" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E781" t="n">
         <v>52.25</v>
@@ -24956,14 +24960,14 @@
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0030</t>
+          <t>MERRA2-BO-0031</t>
         </is>
       </c>
       <c r="D782" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E782" t="n">
-        <v>52.25</v>
+        <v>52.75</v>
       </c>
       <c r="F782" t="inlineStr"/>
     </row>
@@ -24980,11 +24984,11 @@
       </c>
       <c r="C783" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0031</t>
+          <t>MERRA2-BO-0032</t>
         </is>
       </c>
       <c r="D783" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E783" t="n">
         <v>52.75</v>
@@ -25004,11 +25008,11 @@
       </c>
       <c r="C784" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0032</t>
+          <t>MERRA2-BO-0033</t>
         </is>
       </c>
       <c r="D784" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E784" t="n">
         <v>52.75</v>
@@ -25028,11 +25032,11 @@
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0033</t>
+          <t>MERRA2-BO-0034</t>
         </is>
       </c>
       <c r="D785" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E785" t="n">
         <v>52.75</v>
@@ -25052,11 +25056,11 @@
       </c>
       <c r="C786" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0034</t>
+          <t>MERRA2-BO-0035</t>
         </is>
       </c>
       <c r="D786" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E786" t="n">
         <v>52.75</v>
@@ -25076,11 +25080,11 @@
       </c>
       <c r="C787" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0035</t>
+          <t>MERRA2-BO-0036</t>
         </is>
       </c>
       <c r="D787" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E787" t="n">
         <v>52.75</v>
@@ -25100,14 +25104,14 @@
       </c>
       <c r="C788" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0036</t>
+          <t>MERRA2-BO-0037</t>
         </is>
       </c>
       <c r="D788" t="n">
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
       <c r="E788" t="n">
-        <v>52.75</v>
+        <v>53.25</v>
       </c>
       <c r="F788" t="inlineStr"/>
     </row>
@@ -25124,11 +25128,11 @@
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0037</t>
+          <t>MERRA2-BO-0038</t>
         </is>
       </c>
       <c r="D789" t="n">
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
       <c r="E789" t="n">
         <v>53.25</v>
@@ -25148,11 +25152,11 @@
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0038</t>
+          <t>MERRA2-BO-0039</t>
         </is>
       </c>
       <c r="D790" t="n">
-        <v>2.1875</v>
+        <v>2.8125</v>
       </c>
       <c r="E790" t="n">
         <v>53.25</v>
@@ -25172,11 +25176,11 @@
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0039</t>
+          <t>MERRA2-BO-0040</t>
         </is>
       </c>
       <c r="D791" t="n">
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
       <c r="E791" t="n">
         <v>53.25</v>
@@ -25196,11 +25200,11 @@
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0040</t>
+          <t>MERRA2-BO-0041</t>
         </is>
       </c>
       <c r="D792" t="n">
-        <v>3.4375</v>
+        <v>4.0625</v>
       </c>
       <c r="E792" t="n">
         <v>53.25</v>
@@ -25220,40 +25224,16 @@
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>MERRA2-BO-0041</t>
+          <t>MERRA2-BO-0042</t>
         </is>
       </c>
       <c r="D793" t="n">
-        <v>4.0625</v>
+        <v>4.6875</v>
       </c>
       <c r="E793" t="n">
         <v>53.25</v>
       </c>
       <c r="F793" t="inlineStr"/>
-    </row>
-    <row r="794">
-      <c r="A794" t="inlineStr">
-        <is>
-          <t>Borssele Wind</t>
-        </is>
-      </c>
-      <c r="B794" t="inlineStr">
-        <is>
-          <t>MERRA2</t>
-        </is>
-      </c>
-      <c r="C794" t="inlineStr">
-        <is>
-          <t>MERRA2-BO-0042</t>
-        </is>
-      </c>
-      <c r="D794" t="n">
-        <v>4.6875</v>
-      </c>
-      <c r="E794" t="n">
-        <v>53.25</v>
-      </c>
-      <c r="F794" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26455,7 +26435,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Toggle the reference point on/off. Its name/lon/lat come from each farm's own dataset="reference" row in the grid_cells sheet, not from settings -- see settings_advanced for its marker/color/size styling.</t>
+          <t>Toggle the reference point on/off. Its name/lon/lat are found automatically from the matching farm in the wind_farms sheet -- or from a dataset="reference" row in grid_cells, if you want it somewhere else. See settings_advanced for its marker/color/size styling.</t>
         </is>
       </c>
     </row>

</xml_diff>